<commit_message>
Automate generation, editing, and upload of Cars #93, #94, and #95
</commit_message>
<xml_diff>
--- a/100_popular_cars_tracker.xlsx
+++ b/100_popular_cars_tracker.xlsx
@@ -563,7 +563,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Generated &amp; Maintained by Automated Pipeline | Last Updated: 2026-09-17 03:52:52</t>
+          <t>Generated &amp; Maintained by Automated Pipeline | Last Updated: 2026-09-19 03:52:36</t>
         </is>
       </c>
     </row>
@@ -598,17 +598,17 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>90 (90%)</t>
+          <t>95 (95%)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>90 (90%)</t>
+          <t>95 (95%)</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>90 (90%)</t>
+          <t>95 (95%)</t>
         </is>
       </c>
     </row>
@@ -5174,24 +5174,24 @@
           <t>Skoda Slavia</t>
         </is>
       </c>
-      <c r="D99" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E99" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F99" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G99" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G99" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H99" s="9" t="inlineStr">
@@ -5206,12 +5206,12 @@
       </c>
       <c r="J99" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K99" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_91_Skoda_Slavia\Skoda_Slavia.mp4</t>
+        </is>
+      </c>
+      <c r="K99" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5224,24 +5224,24 @@
           <t>Skoda Kushaq</t>
         </is>
       </c>
-      <c r="D100" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E100" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F100" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G100" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D100" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F100" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G100" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H100" s="9" t="inlineStr">
@@ -5256,12 +5256,12 @@
       </c>
       <c r="J100" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K100" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_92_Skoda_Kushaq\Skoda_Kushaq.mp4</t>
+        </is>
+      </c>
+      <c r="K100" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5274,24 +5274,24 @@
           <t>Skoda Kodiaq</t>
         </is>
       </c>
-      <c r="D101" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E101" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F101" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G101" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G101" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H101" s="9" t="inlineStr">
@@ -5306,12 +5306,12 @@
       </c>
       <c r="J101" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K101" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_93_Skoda_Kodiaq\Skoda_Kodiaq.mp4</t>
+        </is>
+      </c>
+      <c r="K101" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5324,24 +5324,24 @@
           <t>Skoda Superb</t>
         </is>
       </c>
-      <c r="D102" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E102" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F102" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G102" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D102" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F102" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G102" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H102" s="9" t="inlineStr">
@@ -5356,12 +5356,12 @@
       </c>
       <c r="J102" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K102" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_94_Skoda_Superb\Skoda_Superb.mp4</t>
+        </is>
+      </c>
+      <c r="K102" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5374,24 +5374,24 @@
           <t>MG Hector</t>
         </is>
       </c>
-      <c r="D103" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E103" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F103" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G103" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D103" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F103" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G103" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H103" s="9" t="inlineStr">
@@ -5406,12 +5406,12 @@
       </c>
       <c r="J103" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K103" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_95_MG_Hector\MG_Hector.mp4</t>
+        </is>
+      </c>
+      <c r="K103" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5757,6 +5757,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K96" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K100" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId95"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update tracker progress: Cars #96, #97, and #98 generated, edited, and published
</commit_message>
<xml_diff>
--- a/100_popular_cars_tracker.xlsx
+++ b/100_popular_cars_tracker.xlsx
@@ -563,7 +563,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Generated &amp; Maintained by Automated Pipeline | Last Updated: 2026-09-19 03:52:36</t>
+          <t>Generated &amp; Maintained by Automated Pipeline | Last Updated: 2026-09-20 01:01:45</t>
         </is>
       </c>
     </row>
@@ -598,17 +598,17 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>95 (95%)</t>
+          <t>98 (98%)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>95 (95%)</t>
+          <t>98 (98%)</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>95 (95%)</t>
+          <t>98 (98%)</t>
         </is>
       </c>
     </row>
@@ -5424,24 +5424,24 @@
           <t>MG Astor</t>
         </is>
       </c>
-      <c r="D104" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E104" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F104" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G104" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D104" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E104" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F104" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G104" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H104" s="9" t="inlineStr">
@@ -5456,12 +5456,12 @@
       </c>
       <c r="J104" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K104" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_96_MG_Astor\MG_Astor.mp4</t>
+        </is>
+      </c>
+      <c r="K104" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5474,24 +5474,24 @@
           <t>Mahindra Scorpio Classic</t>
         </is>
       </c>
-      <c r="D105" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E105" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F105" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G105" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F105" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G105" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H105" s="9" t="inlineStr">
@@ -5506,12 +5506,12 @@
       </c>
       <c r="J105" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K105" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_97_Mahindra_Scorpio_Classic\Mahindra_Scorpio_Classic.mp4</t>
+        </is>
+      </c>
+      <c r="K105" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5524,24 +5524,24 @@
           <t>Hyundai Grand i10 Nios</t>
         </is>
       </c>
-      <c r="D106" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E106" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F106" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G106" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D106" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F106" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G106" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H106" s="9" t="inlineStr">
@@ -5556,12 +5556,12 @@
       </c>
       <c r="J106" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K106" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_98_Hyundai_Grand_i10_Nios\Hyundai_Grand_i10_Nios.mp4</t>
+        </is>
+      </c>
+      <c r="K106" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5762,6 +5762,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId98"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete 100 Popular Cars in India series: 100/100 generated, edited, and uploaded
</commit_message>
<xml_diff>
--- a/100_popular_cars_tracker.xlsx
+++ b/100_popular_cars_tracker.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,13 +76,8 @@
       <sz val="10"/>
       <u val="single"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="007F6000"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -105,12 +100,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -140,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -166,9 +155,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -563,7 +549,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Generated &amp; Maintained by Automated Pipeline | Last Updated: 2026-09-20 01:21:14</t>
+          <t>Generated &amp; Maintained by Automated Pipeline | Last Updated: 2026-09-21 00:30:23</t>
         </is>
       </c>
     </row>
@@ -598,17 +584,17 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>98 (98%)</t>
+          <t>100 (100%)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>98 (98%)</t>
+          <t>100 (100%)</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>98 (98%)</t>
+          <t>100 (100%)</t>
         </is>
       </c>
     </row>
@@ -5574,24 +5560,24 @@
           <t>MG ZS EV</t>
         </is>
       </c>
-      <c r="D107" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E107" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F107" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G107" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D107" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E107" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F107" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G107" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H107" s="9" t="inlineStr">
@@ -5606,12 +5592,12 @@
       </c>
       <c r="J107" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K107" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_99_MG_ZS_EV\MG_ZS_EV.mp4</t>
+        </is>
+      </c>
+      <c r="K107" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5624,24 +5610,24 @@
           <t>Jeep Compass</t>
         </is>
       </c>
-      <c r="D108" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="E108" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="F108" s="11" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G108" s="11" t="inlineStr">
-        <is>
-          <t>Pending Generation</t>
+      <c r="D108" s="8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>EDITED</t>
+        </is>
+      </c>
+      <c r="F108" s="8" t="inlineStr">
+        <is>
+          <t>UPLOADED</t>
+        </is>
+      </c>
+      <c r="G108" s="8" t="inlineStr">
+        <is>
+          <t>Published on YouTube</t>
         </is>
       </c>
       <c r="H108" s="9" t="inlineStr">
@@ -5656,12 +5642,12 @@
       </c>
       <c r="J108" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K108" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>output\100_popular_cars_in_India_100_Jeep_Compass\Jeep_Compass.mp4</t>
+        </is>
+      </c>
+      <c r="K108" s="10" t="inlineStr">
+        <is>
+          <t>https://studio.youtube.com/channel/videos/short</t>
         </is>
       </c>
     </row>
@@ -5765,6 +5751,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K107" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>